<commit_message>
Include entry and exit premium prices for both legs in daily reports
</commit_message>
<xml_diff>
--- a/reports/Daily_Report_2026-05-24.xlsx
+++ b/reports/Daily_Report_2026-05-24.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="Rs. #,##0.00"/>
-    <numFmt numFmtId="166" formatCode="$0.0000"/>
+    <numFmt numFmtId="166" formatCode="$0.00"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
   <fonts count="8">
@@ -515,16 +515,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -537,7 +541,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated on 2026-05-24 13:30:41 IST</t>
+          <t>Generated on 2026-05-24 13:41:22 IST</t>
         </is>
       </c>
     </row>
@@ -556,7 +560,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -578,7 +582,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>184.7547949112889</v>
+        <v>184.9133274463874</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -588,7 +592,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>15334.64797763697</v>
+        <v>15347.80617805015</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -653,20 +657,40 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
+          <t>Call Entry $</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Call Exit $</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
           <t>Put Strike</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>Entry Premium</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Put Entry $</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Put Exit $</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>Total Premium</t>
+        </is>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
         <is>
           <t>P&amp;L (USD)</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="K14" s="9" t="inlineStr">
         <is>
           <t>Exit Reason</t>
         </is>
@@ -688,18 +712,30 @@
           <t>C-BTC-77600-250526</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>P-BTC-75600-250526</t>
         </is>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="G15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="10" t="n">
         <v>37070.90576769917</v>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="J15" s="11" t="n">
         <v>184.6328556991721</v>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>EOD Square-off</t>
         </is>
@@ -721,92 +757,149 @@
           <t>C-BTC-77600-250526</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>P-BTC-75600-250526</t>
         </is>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="G16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="10" t="n">
         <v>35.27025600411677</v>
       </c>
-      <c r="F16" s="11" t="n">
+      <c r="J16" s="11" t="n">
         <v>0.1219392121167715</v>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>EOD Square-off</t>
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-24T13:41:18.178736+05:30</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-24T13:41:22.015811+05:30</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>C-BTC-77600-250526</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>194.1097829472365</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>192.87253053</v>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>P-BTC-75800-250526</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>199.940628953749</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>199.59255602</v>
+      </c>
+      <c r="I17" s="10" t="n">
+        <v>39.40504119009855</v>
+      </c>
+      <c r="J17" s="11" t="n">
+        <v>0.1585325350985514</v>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>EOD Square-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Risk &amp; Market Metrics</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Daily Loss Limit Hit</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>SL Hits</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="n">
-        <v>0</v>
+          <t>Daily Loss Limit Hit</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Hedging Activity</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+          <t>SL Hits</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>ADX Value</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="n">
-        <v>0</v>
+          <t>Hedging Activity</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>IV Level</t>
-        </is>
-      </c>
-      <c r="B23" s="13" t="n">
-        <v>0.432641549789604</v>
+          <t>ADX Value</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t>IV Level</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>0.4313145430816832</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
           <t>High Impact News</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>

</xml_diff>

<commit_message>
Fix force strangle entry instant square-off bug
</commit_message>
<xml_diff>
--- a/reports/Daily_Report_2026-05-24.xlsx
+++ b/reports/Daily_Report_2026-05-24.xlsx
@@ -515,17 +515,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
@@ -541,7 +541,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated on 2026-05-24 13:41:22 IST</t>
+          <t>Generated on 2026-05-24 14:03:33 IST</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>184.9133274463874</v>
+        <v>303.4301022337173</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>15347.80617805015</v>
+        <v>25184.69848539854</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -603,7 +603,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>58.73%</t>
+          <t>58.24%</t>
         </is>
       </c>
     </row>
@@ -831,75 +831,120 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-24T14:03:28.523679+05:30</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-24T14:03:32.948985+05:30</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>C-BTC-84000-260626</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>888.8215265768865</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>888.8215265768865</v>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>P-BTC-76000-290526</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>299.062693556413</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>299.062693556413</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>118.7884220133299</v>
+      </c>
+      <c r="J18" s="11" t="n">
+        <v>118.51677478733</v>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>EOD Square-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Risk &amp; Market Metrics</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Daily Loss Limit Hit</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>SL Hits</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="n">
-        <v>0</v>
+          <t>Daily Loss Limit Hit</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Hedging Activity</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+          <t>SL Hits</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>ADX Value</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="n">
-        <v>0</v>
+          <t>Hedging Activity</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>IV Level</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="n">
-        <v>0.4313145430816832</v>
+          <t>ADX Value</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
+          <t>IV Level</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>0.4112325079030144</v>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
           <t>High Impact News</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>

</xml_diff>